<commit_message>
fix(pricing): Making Class 최소인원 2→3 반영 (PRD 5.2 정합)
- 시트5 C25 라벨 최소 2명→3명
- C26/C28/C29/C32 곱셈·나눗셈 인자 2→3 (매출·소모품·수수료·1인당마진)
- 결과: 최소 시나리오 세션마진 284,640 / 마진율 63.3% / 1인당 94,880 / 소모품 -15,000
- 최대 15명 불변(매출 2,250,000 / 마진 1,945,440)
- 시트5 한정, 기존 GREEN 5값(Dia 267440·Prem 723440·고정비 3452000·손익분기 13) 불변
- soffice 재계산 검증 완료
</commit_message>
<xml_diff>
--- a/KING_STUDIO_Pricing_Model.xlsx
+++ b/KING_STUDIO_Pricing_Model.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:B38"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -823,6 +823,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="50" t="inlineStr">
         <is>
@@ -844,6 +845,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="47">
       <c r="B8" s="50" t="inlineStr">
         <is>
@@ -872,6 +874,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="16.5" customHeight="1" s="47">
       <c r="B13" s="50" t="inlineStr">
         <is>
@@ -900,6 +903,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="47">
       <c r="B18" s="50" t="inlineStr">
         <is>
@@ -935,6 +939,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="16.5" customHeight="1" s="47">
       <c r="B24" s="52" t="inlineStr">
         <is>
@@ -970,6 +975,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="16.5" customHeight="1" s="47">
       <c r="B30" s="50" t="inlineStr">
         <is>
@@ -1012,6 +1018,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="47">
       <c r="B37" s="53" t="inlineStr">
         <is>
@@ -1039,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:E48"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -1063,6 +1070,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="47">
       <c r="B4" s="54" t="inlineStr">
         <is>
@@ -1762,20 +1770,20 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="46" t="inlineStr">
         <is>
           <t>수정·보정비 / 세션 (Dia·Prem)</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="46" t="inlineStr">
         <is>
           <t>KRW</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="46" t="inlineStr">
         <is>
           <t>입력: Dia·Prem 추가 수정작업 (Gold 제외)</t>
         </is>
@@ -1909,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:G40"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -1932,6 +1940,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="68" t="inlineStr">
         <is>
@@ -2394,6 +2403,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="B27" s="49" t="inlineStr">
         <is>
@@ -2401,6 +2411,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="77" t="inlineStr">
         <is>
@@ -2582,6 +2593,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="B38" s="78" t="inlineStr">
         <is>
@@ -2616,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:F13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -2639,6 +2651,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="68" t="inlineStr">
         <is>
@@ -2805,6 +2818,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="47">
       <c r="B12" s="53" t="inlineStr">
         <is>
@@ -2832,7 +2846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:E21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -2856,6 +2870,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="63" t="inlineStr">
         <is>
@@ -2872,6 +2887,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="16.5" customHeight="1" s="47">
       <c r="B6" s="52" t="inlineStr">
         <is>
@@ -2918,6 +2934,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1" s="47">
       <c r="B11" s="52" t="inlineStr">
         <is>
@@ -3017,6 +3034,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="47">
       <c r="B20" s="53" t="inlineStr">
         <is>
@@ -3340,7 +3358,7 @@
       </c>
       <c r="C25" s="89" t="inlineStr">
         <is>
-          <t>최소 2명</t>
+          <t>최소 3명</t>
         </is>
       </c>
       <c r="D25" s="89" t="inlineStr">
@@ -3356,7 +3374,7 @@
         </is>
       </c>
       <c r="C26" s="70">
-        <f>'1.입력값'!$C$11*2</f>
+        <f>'1.입력값'!$C$11*3</f>
         <v/>
       </c>
       <c r="D26" s="70">
@@ -3386,7 +3404,7 @@
         </is>
       </c>
       <c r="C28" s="70">
-        <f>-'1.입력값'!$C$47*2</f>
+        <f>-'1.입력값'!$C$47*3</f>
         <v/>
       </c>
       <c r="D28" s="70">
@@ -3401,7 +3419,7 @@
         </is>
       </c>
       <c r="C29" s="70">
-        <f>-('1.입력값'!$C$11*2*'1.입력값'!$C$27+'1.입력값'!$C$28)</f>
+        <f>-('1.입력값'!$C$11*3*'1.입력값'!$C$27+'1.입력값'!$C$28)</f>
         <v/>
       </c>
       <c r="D29" s="70">
@@ -3446,7 +3464,7 @@
         </is>
       </c>
       <c r="C32" s="71">
-        <f>C30/2</f>
+        <f>C30/3</f>
         <v/>
       </c>
       <c r="D32" s="71">

</xml_diff>

<commit_message>
fix(pricing): 인원별 마진 블록 주석 PRD 5.2 정합 (부채 A)
- 시트2 B39 거짓 일반화 제거: 구 'Gold·Premium도 동일 공식(5인)' → Diamond·Premium 최대 5인, Gold 최대 2인 (PRD 5.2 C10)
- 블록(C32:C36)은 Diamond 예시로 명시 (B30 헤더와 정합, PRD 인당+50% 선형 공식 근거)
- 주석 단일 셀 교체, 수식·숫자 무변경
- 검증: GREEN 5값(Dia 267440·Prem 723440·고정비 3452000·손익분기 13·Gold 241840) 불변, D 커밋값(Making 3명/284640/94880) 불변, soffice 재계산 일치
</commit_message>
<xml_diff>
--- a/KING_STUDIO_Pricing_Model.xlsx
+++ b/KING_STUDIO_Pricing_Model.xlsx
@@ -1917,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="B1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -1940,7 +1940,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="68" t="inlineStr">
         <is>
@@ -2403,7 +2402,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="B27" s="49" t="inlineStr">
         <is>
@@ -2411,7 +2409,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="B29" s="77" t="inlineStr">
         <is>
@@ -2593,7 +2590,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="B38" s="78" t="inlineStr">
         <is>
@@ -2604,7 +2600,7 @@
     <row r="39">
       <c r="B39" s="78" t="inlineStr">
         <is>
-          <t>※ 인원↑ 시 매출은 선형 증가·원가는 거의 고정이라 마진율 상승(5인 최대). Gold·Premium도 동일 공식.</t>
+          <t>※ 인원↑ 시 매출 선형 증가·원가 거의 고정이라 마진율 상승. Diamond·Premium 최대 5인, Gold 최대 2인 (PRD §5.2 C10). 위 블록은 Diamond 예시.</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:E36"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -3085,6 +3081,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="17.15" customHeight="1" s="47">
       <c r="B4" s="88" t="inlineStr">
         <is>
@@ -3214,6 +3211,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="17.15" customHeight="1" s="47">
       <c r="B14" s="88" t="inlineStr">
         <is>
@@ -3343,6 +3341,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="17.15" customHeight="1" s="47">
       <c r="B24" s="55" t="inlineStr">
         <is>
@@ -3472,6 +3471,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="47">
       <c r="B34" s="87" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(pricing): drop duplicate per-headcount summary block (B29:E40), add 3-5p logic note B28 — debt B/A/C10 real fix
</commit_message>
<xml_diff>
--- a/KING_STUDIO_Pricing_Model.xlsx
+++ b/KING_STUDIO_Pricing_Model.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="B1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -823,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="50" t="inlineStr">
         <is>
@@ -845,7 +844,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="47">
       <c r="B8" s="50" t="inlineStr">
         <is>
@@ -874,7 +872,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="16.5" customHeight="1" s="47">
       <c r="B13" s="50" t="inlineStr">
         <is>
@@ -903,7 +900,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="47">
       <c r="B18" s="50" t="inlineStr">
         <is>
@@ -939,7 +935,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="16.5" customHeight="1" s="47">
       <c r="B24" s="52" t="inlineStr">
         <is>
@@ -975,7 +970,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="16.5" customHeight="1" s="47">
       <c r="B30" s="50" t="inlineStr">
         <is>
@@ -1018,7 +1012,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="47">
       <c r="B37" s="53" t="inlineStr">
         <is>
@@ -1046,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="B1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -1070,7 +1063,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="47">
       <c r="B4" s="54" t="inlineStr">
         <is>
@@ -2409,41 +2401,24 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>※ 3~5인 마진 별도 산출 안함. 최저마진은 1인, 전 패키지 +. Gold PRD 5.2 최대 2인.</t>
+        </is>
+      </c>
+    </row>
     <row r="29">
-      <c r="B29" s="77" t="inlineStr">
-        <is>
-          <t>【 인원별 마진 요약 (인당 +50% 정책, C10) 】</t>
-        </is>
-      </c>
+      <c r="B29" s="77" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="78" t="inlineStr">
-        <is>
-          <t>(Diamond 기준 예시 — 매출=정가×배수, 인건비 고정·소모품 인원비례)</t>
-        </is>
-      </c>
+      <c r="B30" s="78" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="79" t="inlineStr">
-        <is>
-          <t>인원</t>
-        </is>
-      </c>
-      <c r="C31" s="79" t="inlineStr">
-        <is>
-          <t>매출(총액)</t>
-        </is>
-      </c>
-      <c r="D31" s="79" t="inlineStr">
-        <is>
-          <t>마진(총액)</t>
-        </is>
-      </c>
-      <c r="E31" s="79" t="inlineStr">
-        <is>
-          <t>마진율</t>
-        </is>
-      </c>
+      <c r="B31" s="79" t="n"/>
+      <c r="C31" s="79" t="n"/>
+      <c r="D31" s="79" t="n"/>
+      <c r="E31" s="79" t="n"/>
       <c r="F31" s="79" t="inlineStr">
         <is>
           <t>1인당 마진</t>
@@ -2456,23 +2431,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="80" t="inlineStr">
-        <is>
-          <t>1인</t>
-        </is>
-      </c>
-      <c r="C32" s="81">
-        <f>$D$5*1.0</f>
-        <v/>
-      </c>
-      <c r="D32" s="82">
-        <f>C32+G32-C32*0.044</f>
-        <v/>
-      </c>
-      <c r="E32" s="83">
-        <f>IF(C32=0,0,D32/C32)</f>
-        <v/>
-      </c>
+      <c r="B32" s="80" t="n"/>
+      <c r="C32" s="81" t="n"/>
+      <c r="D32" s="82" t="n"/>
+      <c r="E32" s="83" t="n"/>
       <c r="F32" s="82">
         <f>D32/1</f>
         <v/>
@@ -2483,23 +2445,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="80" t="inlineStr">
-        <is>
-          <t>2인</t>
-        </is>
-      </c>
-      <c r="C33" s="81">
-        <f>$D$5*1.5</f>
-        <v/>
-      </c>
-      <c r="D33" s="82">
-        <f>C33+G33-C33*0.044</f>
-        <v/>
-      </c>
-      <c r="E33" s="83">
-        <f>IF(C33=0,0,D33/C33)</f>
-        <v/>
-      </c>
+      <c r="B33" s="80" t="n"/>
+      <c r="C33" s="81" t="n"/>
+      <c r="D33" s="82" t="n"/>
+      <c r="E33" s="83" t="n"/>
       <c r="F33" s="82">
         <f>D33/2</f>
         <v/>
@@ -2510,23 +2459,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="80" t="inlineStr">
-        <is>
-          <t>3인</t>
-        </is>
-      </c>
-      <c r="C34" s="81">
-        <f>$D$5*2.0</f>
-        <v/>
-      </c>
-      <c r="D34" s="82">
-        <f>C34+G34-C34*0.044</f>
-        <v/>
-      </c>
-      <c r="E34" s="83">
-        <f>IF(C34=0,0,D34/C34)</f>
-        <v/>
-      </c>
+      <c r="B34" s="80" t="n"/>
+      <c r="C34" s="81" t="n"/>
+      <c r="D34" s="82" t="n"/>
+      <c r="E34" s="83" t="n"/>
       <c r="F34" s="82">
         <f>D34/3</f>
         <v/>
@@ -2537,23 +2473,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="80" t="inlineStr">
-        <is>
-          <t>4인</t>
-        </is>
-      </c>
-      <c r="C35" s="81">
-        <f>$D$5*2.5</f>
-        <v/>
-      </c>
-      <c r="D35" s="82">
-        <f>C35+G35-C35*0.044</f>
-        <v/>
-      </c>
-      <c r="E35" s="83">
-        <f>IF(C35=0,0,D35/C35)</f>
-        <v/>
-      </c>
+      <c r="B35" s="80" t="n"/>
+      <c r="C35" s="81" t="n"/>
+      <c r="D35" s="82" t="n"/>
+      <c r="E35" s="83" t="n"/>
       <c r="F35" s="82">
         <f>D35/4</f>
         <v/>
@@ -2564,23 +2487,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="80" t="inlineStr">
-        <is>
-          <t>5인</t>
-        </is>
-      </c>
-      <c r="C36" s="81">
-        <f>$D$5*3.0</f>
-        <v/>
-      </c>
-      <c r="D36" s="82">
-        <f>C36+G36-C36*0.044</f>
-        <v/>
-      </c>
-      <c r="E36" s="83">
-        <f>IF(C36=0,0,D36/C36)</f>
-        <v/>
-      </c>
+      <c r="B36" s="80" t="n"/>
+      <c r="C36" s="81" t="n"/>
+      <c r="D36" s="82" t="n"/>
+      <c r="E36" s="83" t="n"/>
       <c r="F36" s="82">
         <f>D36/5</f>
         <v/>
@@ -2590,26 +2500,15 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
-      <c r="B38" s="78" t="inlineStr">
-        <is>
-          <t>※ 공식: 매출=정가×(1+0.5×(인원−1)). 인건비·통역·믹싱·MV·촬영은 1팀 고정, 소모품만 인원비례.</t>
-        </is>
-      </c>
+      <c r="B38" s="78" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="78" t="inlineStr">
-        <is>
-          <t>※ 인원↑ 시 매출 선형 증가·원가 거의 고정이라 마진율 상승. Diamond·Premium 최대 5인, Gold 최대 2인 (PRD §5.2 C10). 위 블록은 Diamond 예시.</t>
-        </is>
-      </c>
+      <c r="B39" s="78" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="78" t="inlineStr">
-        <is>
-          <t>※ 결제수수료는 PayPal 4.4% 근사(고정수수료 제외, 요약용). 정밀 계산은 상단 1·2인 블록 참조.</t>
-        </is>
-      </c>
+      <c r="B40" s="78" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2624,7 +2523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="B1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -2647,7 +2546,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="68" t="inlineStr">
         <is>
@@ -2814,7 +2712,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="47">
       <c r="B12" s="53" t="inlineStr">
         <is>
@@ -2842,7 +2739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="B1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -2866,7 +2763,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="47">
       <c r="B4" s="63" t="inlineStr">
         <is>
@@ -2883,7 +2779,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="16.5" customHeight="1" s="47">
       <c r="B6" s="52" t="inlineStr">
         <is>
@@ -2930,7 +2825,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1" s="47">
       <c r="B11" s="52" t="inlineStr">
         <is>
@@ -3030,7 +2924,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="47">
       <c r="B20" s="53" t="inlineStr">
         <is>
@@ -3058,7 +2951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="B1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="46" min="1" max="1"/>
@@ -3081,7 +2974,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="17.15" customHeight="1" s="47">
       <c r="B4" s="88" t="inlineStr">
         <is>
@@ -3211,7 +3103,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="17.15" customHeight="1" s="47">
       <c r="B14" s="88" t="inlineStr">
         <is>
@@ -3341,7 +3232,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="17.15" customHeight="1" s="47">
       <c r="B24" s="55" t="inlineStr">
         <is>
@@ -3471,7 +3361,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="47">
       <c r="B34" s="87" t="inlineStr">
         <is>

</xml_diff>